<commit_message>
Add Kerki #42: RoundNzt takes a second Season 4 win
Kerki #42 (2026-09-20), maps Symetra by Shadynook, Vaporwave Valley by
IronDragon111000 and Ferret Found Magnets by variableferret.

Winners: RoundNzt, Kernkob, ZOMAN, microways, tatari_lover2008.
Finalists: Lexer, brrryy. 27 others, 34 in the lobby.
Nuisance: justMaki (tested all three maps) plus Shadynook and
IronDragon111000, both map authors who raced.

Clean capture, 15 scoring rounds, no gaps. Parsed with --no-warmup:
the Top->Out tournament mod scores every round from the first, so v2
cups have no discovery rounds. The default warmup logic gave 3 winners
against the tracker's 5; --no-warmup reproduces the tracker exactly,
including the 5th win landing in the last played round, which is what
ended the tournament.

Tommygaming and Victor both crossed 1000 in that final round. The
last-round rule keeps them out of the finalist list, so they sit in
Others at 1000.

RoundNzt now leads Season 4 on 400 from two first-place wins.
</commit_message>
<xml_diff>
--- a/Kerki Comp Results 31+.xlsx
+++ b/Kerki Comp Results 31+.xlsx
@@ -3973,7 +3973,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C59"/>
+  <dimension ref="A1:I59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3982,6 +3982,11 @@
           <t>6/9/26</t>
         </is>
       </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>20/9/26</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3989,6 +3994,11 @@
           <t>Kerki Comp #41 - Maps by DeeDeeNaNaNa, PlusMicron, Kernkob &amp; Maki</t>
         </is>
       </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Kerki Comp #42 - Maps by Shadynook, IronDragon111000, variableferret</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -4006,9 +4016,29 @@
           <t>Points</t>
         </is>
       </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Placement</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Points</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
+        <is>
+          <t>Winners</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
         <is>
           <t>Winners</t>
         </is>
@@ -4023,6 +4053,14 @@
           <t>RoundNzt</t>
         </is>
       </c>
+      <c r="G5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>RoundNzt</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -4033,6 +4071,14 @@
           <t>Quickracer10</t>
         </is>
       </c>
+      <c r="G6" t="n">
+        <v>2</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Kernkob</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -4043,6 +4089,14 @@
           <t>PandaMane</t>
         </is>
       </c>
+      <c r="G7" t="n">
+        <v>3</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>ZOMAN</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -4053,6 +4107,14 @@
           <t>Lexer</t>
         </is>
       </c>
+      <c r="G8" t="n">
+        <v>4</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>microways</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -4063,9 +4125,22 @@
           <t>Minkus</t>
         </is>
       </c>
+      <c r="G9" t="n">
+        <v>5</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>tatari_lover2008</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
+        <is>
+          <t>Finalists</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
         <is>
           <t>Finalists</t>
         </is>
@@ -4080,6 +4155,14 @@
           <t>Jake</t>
         </is>
       </c>
+      <c r="G11" t="n">
+        <v>1</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Lexer</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -4090,6 +4173,14 @@
           <t>Murrl</t>
         </is>
       </c>
+      <c r="G12" t="n">
+        <v>2</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>brrryy</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -4100,6 +4191,11 @@
           <t>Eclipse135</t>
         </is>
       </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -4110,12 +4206,34 @@
           <t>agix</t>
         </is>
       </c>
+      <c r="G14" t="n">
+        <v>1</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Tommygaming</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>1000</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
           <t>Other</t>
         </is>
+      </c>
+      <c r="G15" t="n">
+        <v>2</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Victor</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>1000</v>
       </c>
     </row>
     <row r="16">
@@ -4130,6 +4248,17 @@
       <c r="C16" t="n">
         <v>950</v>
       </c>
+      <c r="G16" t="n">
+        <v>3</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Minkus</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>958</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -4143,6 +4272,17 @@
       <c r="C17" t="n">
         <v>865</v>
       </c>
+      <c r="G17" t="n">
+        <v>4</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Warsnac</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
+        <v>903</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -4156,6 +4296,17 @@
       <c r="C18" t="n">
         <v>805</v>
       </c>
+      <c r="G18" t="n">
+        <v>5</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>redal</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>790</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -4169,6 +4320,17 @@
       <c r="C19" t="n">
         <v>771</v>
       </c>
+      <c r="G19" t="n">
+        <v>6</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Revenger_19</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
+        <v>779</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -4182,6 +4344,17 @@
       <c r="C20" t="n">
         <v>734</v>
       </c>
+      <c r="G20" t="n">
+        <v>7</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Noxitu</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
+        <v>755</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -4195,6 +4368,17 @@
       <c r="C21" t="n">
         <v>715</v>
       </c>
+      <c r="G21" t="n">
+        <v>8</v>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Heart-TGV</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
+        <v>723</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -4208,6 +4392,17 @@
       <c r="C22" t="n">
         <v>666</v>
       </c>
+      <c r="G22" t="n">
+        <v>9</v>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>MALIYO</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
+        <v>721</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -4221,6 +4416,17 @@
       <c r="C23" t="n">
         <v>665</v>
       </c>
+      <c r="G23" t="n">
+        <v>10</v>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>PlusMicron</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
+        <v>657</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -4234,6 +4440,17 @@
       <c r="C24" t="n">
         <v>661</v>
       </c>
+      <c r="G24" t="n">
+        <v>11</v>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>aizpun</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
+        <v>652</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -4247,6 +4464,17 @@
       <c r="C25" t="n">
         <v>626</v>
       </c>
+      <c r="G25" t="n">
+        <v>12</v>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Gimpel</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
+        <v>638</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -4260,6 +4488,17 @@
       <c r="C26" t="n">
         <v>619</v>
       </c>
+      <c r="G26" t="n">
+        <v>13</v>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Six</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
+        <v>627</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -4273,6 +4512,17 @@
       <c r="C27" t="n">
         <v>618</v>
       </c>
+      <c r="G27" t="n">
+        <v>14</v>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>wokonbike</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
+        <v>592</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -4286,6 +4536,17 @@
       <c r="C28" t="n">
         <v>617</v>
       </c>
+      <c r="G28" t="n">
+        <v>15</v>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>DeeDeeNaNaNa</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
+        <v>587</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -4299,6 +4560,17 @@
       <c r="C29" t="n">
         <v>591</v>
       </c>
+      <c r="G29" t="n">
+        <v>16</v>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>kentback</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
+        <v>546</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -4312,6 +4584,17 @@
       <c r="C30" t="n">
         <v>576</v>
       </c>
+      <c r="G30" t="n">
+        <v>17</v>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Akane</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
+        <v>531</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -4325,6 +4608,17 @@
       <c r="C31" t="n">
         <v>560</v>
       </c>
+      <c r="G31" t="n">
+        <v>18</v>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>timesprout</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
+        <v>520</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -4338,6 +4632,17 @@
       <c r="C32" t="n">
         <v>557</v>
       </c>
+      <c r="G32" t="n">
+        <v>19</v>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>St Nicholas</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
+        <v>478</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -4351,6 +4656,17 @@
       <c r="C33" t="n">
         <v>521</v>
       </c>
+      <c r="G33" t="n">
+        <v>20</v>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>kkincaid97</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
+        <v>454</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -4364,6 +4680,17 @@
       <c r="C34" t="n">
         <v>496</v>
       </c>
+      <c r="G34" t="n">
+        <v>21</v>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>SjorsTea</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
+        <v>420</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -4377,6 +4704,17 @@
       <c r="C35" t="n">
         <v>485</v>
       </c>
+      <c r="G35" t="n">
+        <v>22</v>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Aurum</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
+        <v>397</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -4390,6 +4728,17 @@
       <c r="C36" t="n">
         <v>408</v>
       </c>
+      <c r="G36" t="n">
+        <v>23</v>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Barn</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
+        <v>340</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -4403,6 +4752,17 @@
       <c r="C37" t="n">
         <v>313</v>
       </c>
+      <c r="G37" t="n">
+        <v>24</v>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>M4DSCOTSM4N</t>
+        </is>
+      </c>
+      <c r="I37" t="n">
+        <v>320</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -4416,6 +4776,17 @@
       <c r="C38" t="n">
         <v>292</v>
       </c>
+      <c r="G38" t="n">
+        <v>25</v>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>DeiRex</t>
+        </is>
+      </c>
+      <c r="I38" t="n">
+        <v>275</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -4429,6 +4800,17 @@
       <c r="C39" t="n">
         <v>236</v>
       </c>
+      <c r="G39" t="n">
+        <v>26</v>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Zeus</t>
+        </is>
+      </c>
+      <c r="I39" t="n">
+        <v>250</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -4442,6 +4824,17 @@
       <c r="C40" t="n">
         <v>202</v>
       </c>
+      <c r="G40" t="n">
+        <v>27</v>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Flinzard</t>
+        </is>
+      </c>
+      <c r="I40" t="n">
+        <v>165</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -4455,12 +4848,28 @@
       <c r="C41" t="n">
         <v>115</v>
       </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Nuisance</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
           <t>Nuisance</t>
         </is>
+      </c>
+      <c r="G42" t="n">
+        <v>1</v>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>justMaki</t>
+        </is>
+      </c>
+      <c r="I42" t="n">
+        <v>747</v>
       </c>
     </row>
     <row r="43">
@@ -4475,6 +4884,17 @@
       <c r="C43" t="n">
         <v>800</v>
       </c>
+      <c r="G43" t="n">
+        <v>2</v>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>IronDragon111000</t>
+        </is>
+      </c>
+      <c r="I43" t="n">
+        <v>588</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -4487,6 +4907,17 @@
       </c>
       <c r="C44" t="n">
         <v>758</v>
+      </c>
+      <c r="G44" t="n">
+        <v>3</v>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Shadynook</t>
+        </is>
+      </c>
+      <c r="I44" t="n">
+        <v>384</v>
       </c>
     </row>
     <row r="45"/>

</xml_diff>